<commit_message>
Fix pricing error + add lean scenario and cash flow chart
Corrected B2B price from 20.41€/h → 22.03€/h (3-employee escandallo).
Previous value was a stale manual estimate; Excel escandallo was always
correct but charts and calculator used wrong figure.

Changes:
- Excel: fixed prices in P&L sheet; new Sheet 6 'CashFlow Lean' with
  progressive hiring (0→1→2→3 employees) comparing full structure
  (1,430€/mo) vs lean (780€/mo: home office + own car)
- Charts: corrected break-even with 22.03€/h; new chart comparing EBITDA
  by occupancy rate (full vs lean); new 18-month progressive cash flow
  chart showing capital needed (13,310€ full / 5,601€ lean)
- Calculator: fixed price hint, added viability reference table

Key findings: lean scenario reaches first positive month at M6 vs M10,
needs 7k€ vs 17k€ capital, recovers investment by M16.

https://claude.ai/code/session_0163DbmQMjco8cNFwnC3Y3UM
</commit_message>
<xml_diff>
--- a/brillopal/BrillOPal_Gestion.xlsx
+++ b/brillopal/BrillOPal_Gestion.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3_Planificación Servicios" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4_Facturación y Cobros" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5_Cuenta Resultados 18M" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6_CashFlow Lean (Recomendado)" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +25,7 @@
     <numFmt numFmtId="164" formatCode="#,##0.00 €"/>
     <numFmt numFmtId="165" formatCode="#,##0.0 &quot;h&quot;"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -68,8 +69,13 @@
       <color rgb="001F3864"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -121,6 +127,11 @@
         <fgColor rgb="00FFCCCC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4C7C3"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -148,7 +159,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -245,6 +256,31 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3317,7 +3353,7 @@
   <dimension ref="A1:BL15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
@@ -3337,7 +3373,7 @@
     <col width="10" customWidth="1" min="18" max="18"/>
     <col width="10" customWidth="1" min="19" max="19"/>
     <col width="10" customWidth="1" min="20" max="20"/>
-    <col width="30" customWidth="1" min="23" max="23"/>
+    <col width="32" customWidth="1" min="23" max="23"/>
     <col width="10" customWidth="1" min="24" max="24"/>
     <col width="10" customWidth="1" min="25" max="25"/>
     <col width="10" customWidth="1" min="26" max="26"/>
@@ -3357,7 +3393,7 @@
     <col width="10" customWidth="1" min="40" max="40"/>
     <col width="10" customWidth="1" min="41" max="41"/>
     <col width="10" customWidth="1" min="42" max="42"/>
-    <col width="30" customWidth="1" min="45" max="45"/>
+    <col width="32" customWidth="1" min="45" max="45"/>
     <col width="10" customWidth="1" min="46" max="46"/>
     <col width="10" customWidth="1" min="47" max="47"/>
     <col width="10" customWidth="1" min="48" max="48"/>
@@ -3382,17 +3418,17 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ESCENARIO 1 EMPLEADO</t>
+          <t>ESCENARIO 1 EMPLEADO – Estructura completa (1.430€/mes)</t>
         </is>
       </c>
       <c r="W1" s="30" t="inlineStr">
         <is>
-          <t>ESCENARIO 3 EMPLEADOS</t>
+          <t>ESCENARIO 3 EMPLEADOS – Estructura completa (1.430€/mes)</t>
         </is>
       </c>
       <c r="AS1" s="31" t="inlineStr">
         <is>
-          <t>ESCENARIO 5 EMPLEADOS</t>
+          <t>ESCENARIO 5 EMPLEADOS – Estructura completa (1.430€/mes)</t>
         </is>
       </c>
     </row>
@@ -4077,377 +4113,377 @@
     <row r="5">
       <c r="A5" s="36" t="inlineStr">
         <is>
-          <t>Ingresos B2B (s/IVA)</t>
+          <t>Ingresos B2B (s/IVA) 22,03€/h</t>
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>703.18828125</v>
+        <v>759.00234375</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>904.09921875</v>
+        <v>975.86015625</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>1105.01015625</v>
+        <v>1192.71796875</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>1305.92109375</v>
+        <v>1409.57578125</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>1406.3765625</v>
+        <v>1518.0046875</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>1446.55875</v>
+        <v>1561.37625</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>1506.83203125</v>
+        <v>1626.43359375</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>1506.83203125</v>
+        <v>1626.43359375</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>1567.1053125</v>
+        <v>1691.4909375</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>1607.2875</v>
+        <v>1734.8625</v>
       </c>
       <c r="L5" s="5" t="n">
-        <v>1647.4696875</v>
+        <v>1778.2340625</v>
       </c>
       <c r="M5" s="5" t="n">
-        <v>1707.74296875</v>
+        <v>1843.29140625</v>
       </c>
       <c r="N5" s="5" t="n">
-        <v>1707.74296875</v>
+        <v>1843.29140625</v>
       </c>
       <c r="O5" s="5" t="n">
-        <v>1647.4696875</v>
+        <v>1778.2340625</v>
       </c>
       <c r="P5" s="5" t="n">
-        <v>1747.92515625</v>
+        <v>1886.66296875</v>
       </c>
       <c r="Q5" s="5" t="n">
-        <v>1768.01625</v>
+        <v>1908.34875</v>
       </c>
       <c r="R5" s="5" t="n">
-        <v>1808.1984375</v>
+        <v>1951.7203125</v>
       </c>
       <c r="S5" s="5" t="n">
-        <v>1808.1984375</v>
+        <v>1951.7203125</v>
       </c>
       <c r="T5" s="39" t="n">
-        <v>26901.97453125</v>
+        <v>29037.26109375</v>
       </c>
       <c r="W5" s="36" t="inlineStr">
         <is>
-          <t>Ingresos B2B (s/IVA)</t>
+          <t>Ingresos B2B (s/IVA) 22,03€/h</t>
         </is>
       </c>
       <c r="X5" s="5" t="n">
-        <v>2109.56484375</v>
+        <v>2277.00703125</v>
       </c>
       <c r="Y5" s="5" t="n">
-        <v>2712.29765625</v>
+        <v>2927.58046875</v>
       </c>
       <c r="Z5" s="5" t="n">
-        <v>3315.03046875</v>
+        <v>3578.15390625</v>
       </c>
       <c r="AA5" s="5" t="n">
-        <v>3917.76328125</v>
+        <v>4228.72734375</v>
       </c>
       <c r="AB5" s="5" t="n">
-        <v>4219.1296875</v>
+        <v>4554.0140625</v>
       </c>
       <c r="AC5" s="5" t="n">
-        <v>4339.67625</v>
+        <v>4684.12875</v>
       </c>
       <c r="AD5" s="5" t="n">
-        <v>4520.49609375</v>
+        <v>4879.30078125</v>
       </c>
       <c r="AE5" s="5" t="n">
-        <v>4520.49609375</v>
+        <v>4879.30078125</v>
       </c>
       <c r="AF5" s="5" t="n">
-        <v>4701.3159375</v>
+        <v>5074.472812499999</v>
       </c>
       <c r="AG5" s="5" t="n">
-        <v>4821.862499999999</v>
+        <v>5204.5875</v>
       </c>
       <c r="AH5" s="5" t="n">
-        <v>4942.4090625</v>
+        <v>5334.7021875</v>
       </c>
       <c r="AI5" s="5" t="n">
-        <v>5123.228906249999</v>
+        <v>5529.874218749999</v>
       </c>
       <c r="AJ5" s="5" t="n">
-        <v>5123.228906249999</v>
+        <v>5529.874218749999</v>
       </c>
       <c r="AK5" s="5" t="n">
-        <v>4942.4090625</v>
+        <v>5334.7021875</v>
       </c>
       <c r="AL5" s="5" t="n">
-        <v>5243.77546875</v>
+        <v>5659.988906250001</v>
       </c>
       <c r="AM5" s="5" t="n">
-        <v>5304.04875</v>
+        <v>5725.04625</v>
       </c>
       <c r="AN5" s="5" t="n">
-        <v>5424.5953125</v>
+        <v>5855.160937500001</v>
       </c>
       <c r="AO5" s="5" t="n">
-        <v>5424.5953125</v>
+        <v>5855.160937500001</v>
       </c>
       <c r="AP5" s="39" t="n">
-        <v>80705.92359374999</v>
+        <v>87111.78328125</v>
       </c>
       <c r="AS5" s="36" t="inlineStr">
         <is>
-          <t>Ingresos B2B (s/IVA)</t>
+          <t>Ingresos B2B (s/IVA) 22,03€/h</t>
         </is>
       </c>
       <c r="AT5" s="5" t="n">
-        <v>3515.94140625</v>
+        <v>3795.01171875</v>
       </c>
       <c r="AU5" s="5" t="n">
-        <v>4520.49609375</v>
+        <v>4879.30078125</v>
       </c>
       <c r="AV5" s="5" t="n">
-        <v>5525.05078125</v>
+        <v>5963.58984375</v>
       </c>
       <c r="AW5" s="5" t="n">
-        <v>6529.60546875</v>
+        <v>7047.87890625</v>
       </c>
       <c r="AX5" s="5" t="n">
-        <v>7031.882812499999</v>
+        <v>7590.023437499999</v>
       </c>
       <c r="AY5" s="5" t="n">
-        <v>7232.79375</v>
+        <v>7806.88125</v>
       </c>
       <c r="AZ5" s="5" t="n">
-        <v>7534.16015625</v>
+        <v>8132.16796875</v>
       </c>
       <c r="BA5" s="5" t="n">
-        <v>7534.16015625</v>
+        <v>8132.16796875</v>
       </c>
       <c r="BB5" s="5" t="n">
-        <v>7835.5265625</v>
+        <v>8457.4546875</v>
       </c>
       <c r="BC5" s="5" t="n">
-        <v>8036.4375</v>
+        <v>8674.3125</v>
       </c>
       <c r="BD5" s="5" t="n">
-        <v>8237.348437500001</v>
+        <v>8891.1703125</v>
       </c>
       <c r="BE5" s="5" t="n">
-        <v>8538.71484375</v>
+        <v>9216.45703125</v>
       </c>
       <c r="BF5" s="5" t="n">
-        <v>8538.71484375</v>
+        <v>9216.45703125</v>
       </c>
       <c r="BG5" s="5" t="n">
-        <v>8237.348437500001</v>
+        <v>8891.1703125</v>
       </c>
       <c r="BH5" s="5" t="n">
-        <v>8739.625781250001</v>
+        <v>9433.31484375</v>
       </c>
       <c r="BI5" s="5" t="n">
-        <v>8840.081249999999</v>
+        <v>9541.74375</v>
       </c>
       <c r="BJ5" s="5" t="n">
-        <v>9040.9921875</v>
+        <v>9758.6015625</v>
       </c>
       <c r="BK5" s="5" t="n">
-        <v>9040.9921875</v>
+        <v>9758.6015625</v>
       </c>
       <c r="BL5" s="39" t="n">
-        <v>134509.87265625</v>
+        <v>145186.30546875</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="36" t="inlineStr">
         <is>
-          <t>Ingresos B2C (s/IVA)</t>
+          <t>Ingresos B2C (s/IVA) 22,22€/h</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>332.2265625</v>
+        <v>331.93125</v>
       </c>
       <c r="C6" s="5" t="n">
-        <v>427.1484375</v>
+        <v>426.76875</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>522.0703125</v>
+        <v>521.60625</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>616.9921875</v>
+        <v>616.44375</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>664.453125</v>
+        <v>663.8625000000001</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>683.4375</v>
+        <v>682.83</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>711.9140625</v>
+        <v>711.28125</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>711.9140625</v>
+        <v>711.28125</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>740.390625</v>
+        <v>739.7325</v>
       </c>
       <c r="K6" s="5" t="n">
-        <v>759.375</v>
+        <v>758.7</v>
       </c>
       <c r="L6" s="5" t="n">
-        <v>778.359375</v>
+        <v>777.6675</v>
       </c>
       <c r="M6" s="5" t="n">
-        <v>806.8359375</v>
+        <v>806.11875</v>
       </c>
       <c r="N6" s="5" t="n">
-        <v>806.8359375</v>
+        <v>806.11875</v>
       </c>
       <c r="O6" s="5" t="n">
-        <v>778.359375</v>
+        <v>777.6675</v>
       </c>
       <c r="P6" s="5" t="n">
-        <v>825.8203125</v>
+        <v>825.0862500000001</v>
       </c>
       <c r="Q6" s="5" t="n">
-        <v>835.3125</v>
+        <v>834.5700000000001</v>
       </c>
       <c r="R6" s="5" t="n">
-        <v>854.296875</v>
+        <v>853.5375</v>
       </c>
       <c r="S6" s="5" t="n">
-        <v>854.296875</v>
+        <v>853.5375</v>
       </c>
       <c r="T6" s="39" t="n">
-        <v>12710.0390625</v>
+        <v>12698.74125</v>
       </c>
       <c r="W6" s="36" t="inlineStr">
         <is>
-          <t>Ingresos B2C (s/IVA)</t>
+          <t>Ingresos B2C (s/IVA) 22,22€/h</t>
         </is>
       </c>
       <c r="X6" s="5" t="n">
-        <v>996.6796875</v>
+        <v>995.79375</v>
       </c>
       <c r="Y6" s="5" t="n">
-        <v>1281.4453125</v>
+        <v>1280.30625</v>
       </c>
       <c r="Z6" s="5" t="n">
-        <v>1566.2109375</v>
+        <v>1564.81875</v>
       </c>
       <c r="AA6" s="5" t="n">
-        <v>1850.9765625</v>
+        <v>1849.33125</v>
       </c>
       <c r="AB6" s="5" t="n">
-        <v>1993.359375</v>
+        <v>1991.5875</v>
       </c>
       <c r="AC6" s="5" t="n">
-        <v>2050.3125</v>
+        <v>2048.49</v>
       </c>
       <c r="AD6" s="5" t="n">
-        <v>2135.7421875</v>
+        <v>2133.84375</v>
       </c>
       <c r="AE6" s="5" t="n">
-        <v>2135.7421875</v>
+        <v>2133.84375</v>
       </c>
       <c r="AF6" s="5" t="n">
-        <v>2221.171875</v>
+        <v>2219.1975</v>
       </c>
       <c r="AG6" s="5" t="n">
-        <v>2278.125</v>
+        <v>2276.1</v>
       </c>
       <c r="AH6" s="5" t="n">
-        <v>2335.078125</v>
+        <v>2333.0025</v>
       </c>
       <c r="AI6" s="5" t="n">
-        <v>2420.5078125</v>
+        <v>2418.35625</v>
       </c>
       <c r="AJ6" s="5" t="n">
-        <v>2420.5078125</v>
+        <v>2418.35625</v>
       </c>
       <c r="AK6" s="5" t="n">
-        <v>2335.078125</v>
+        <v>2333.0025</v>
       </c>
       <c r="AL6" s="5" t="n">
-        <v>2477.4609375</v>
+        <v>2475.25875</v>
       </c>
       <c r="AM6" s="5" t="n">
-        <v>2505.9375</v>
+        <v>2503.71</v>
       </c>
       <c r="AN6" s="5" t="n">
-        <v>2562.890625</v>
+        <v>2560.6125</v>
       </c>
       <c r="AO6" s="5" t="n">
-        <v>2562.890625</v>
+        <v>2560.6125</v>
       </c>
       <c r="AP6" s="39" t="n">
-        <v>38130.1171875</v>
+        <v>38096.22375</v>
       </c>
       <c r="AS6" s="36" t="inlineStr">
         <is>
-          <t>Ingresos B2C (s/IVA)</t>
+          <t>Ingresos B2C (s/IVA) 22,22€/h</t>
         </is>
       </c>
       <c r="AT6" s="5" t="n">
-        <v>1661.1328125</v>
+        <v>1659.65625</v>
       </c>
       <c r="AU6" s="5" t="n">
-        <v>2135.7421875</v>
+        <v>2133.84375</v>
       </c>
       <c r="AV6" s="5" t="n">
-        <v>2610.3515625</v>
+        <v>2608.03125</v>
       </c>
       <c r="AW6" s="5" t="n">
-        <v>3084.9609375</v>
+        <v>3082.21875</v>
       </c>
       <c r="AX6" s="5" t="n">
-        <v>3322.265625</v>
+        <v>3319.3125</v>
       </c>
       <c r="AY6" s="5" t="n">
-        <v>3417.1875</v>
+        <v>3414.15</v>
       </c>
       <c r="AZ6" s="5" t="n">
-        <v>3559.5703125</v>
+        <v>3556.40625</v>
       </c>
       <c r="BA6" s="5" t="n">
-        <v>3559.5703125</v>
+        <v>3556.40625</v>
       </c>
       <c r="BB6" s="5" t="n">
-        <v>3701.953125</v>
+        <v>3698.6625</v>
       </c>
       <c r="BC6" s="5" t="n">
-        <v>3796.875</v>
+        <v>3793.5</v>
       </c>
       <c r="BD6" s="5" t="n">
-        <v>3891.796875</v>
+        <v>3888.3375</v>
       </c>
       <c r="BE6" s="5" t="n">
-        <v>4034.1796875</v>
+        <v>4030.59375</v>
       </c>
       <c r="BF6" s="5" t="n">
-        <v>4034.1796875</v>
+        <v>4030.59375</v>
       </c>
       <c r="BG6" s="5" t="n">
-        <v>3891.796875</v>
+        <v>3888.3375</v>
       </c>
       <c r="BH6" s="5" t="n">
-        <v>4129.1015625</v>
+        <v>4125.43125</v>
       </c>
       <c r="BI6" s="5" t="n">
-        <v>4176.5625</v>
+        <v>4172.85</v>
       </c>
       <c r="BJ6" s="5" t="n">
-        <v>4271.484375</v>
+        <v>4267.6875</v>
       </c>
       <c r="BK6" s="5" t="n">
-        <v>4271.484375</v>
+        <v>4267.6875</v>
       </c>
       <c r="BL6" s="39" t="n">
-        <v>63550.1953125</v>
+        <v>63493.70625</v>
       </c>
     </row>
     <row r="7">
@@ -4457,61 +4493,61 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>1035.41484375</v>
+        <v>1090.93359375</v>
       </c>
       <c r="C7" s="5" t="n">
-        <v>1331.24765625</v>
+        <v>1402.62890625</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>1627.08046875</v>
+        <v>1714.32421875</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>1922.91328125</v>
+        <v>2026.01953125</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>2070.8296875</v>
+        <v>2181.8671875</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>2129.99625</v>
+        <v>2244.20625</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>2218.74609375</v>
+        <v>2337.71484375</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>2218.74609375</v>
+        <v>2337.71484375</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>2307.4959375</v>
+        <v>2431.2234375</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>2366.6625</v>
+        <v>2493.5625</v>
       </c>
       <c r="L7" s="5" t="n">
-        <v>2425.8290625</v>
+        <v>2555.9015625</v>
       </c>
       <c r="M7" s="5" t="n">
-        <v>2514.57890625</v>
+        <v>2649.41015625</v>
       </c>
       <c r="N7" s="5" t="n">
-        <v>2514.57890625</v>
+        <v>2649.41015625</v>
       </c>
       <c r="O7" s="5" t="n">
-        <v>2425.8290625</v>
+        <v>2555.9015625</v>
       </c>
       <c r="P7" s="5" t="n">
-        <v>2573.74546875</v>
+        <v>2711.74921875</v>
       </c>
       <c r="Q7" s="5" t="n">
-        <v>2603.32875</v>
+        <v>2742.91875</v>
       </c>
       <c r="R7" s="5" t="n">
-        <v>2662.4953125</v>
+        <v>2805.2578125</v>
       </c>
       <c r="S7" s="5" t="n">
-        <v>2662.4953125</v>
+        <v>2805.2578125</v>
       </c>
       <c r="T7" s="39" t="n">
-        <v>39612.01359375001</v>
+        <v>41736.00234375</v>
       </c>
       <c r="W7" s="40" t="inlineStr">
         <is>
@@ -4519,61 +4555,61 @@
         </is>
       </c>
       <c r="X7" s="5" t="n">
-        <v>3106.24453125</v>
+        <v>3272.80078125</v>
       </c>
       <c r="Y7" s="5" t="n">
-        <v>3993.74296875</v>
+        <v>4207.88671875</v>
       </c>
       <c r="Z7" s="5" t="n">
-        <v>4881.24140625</v>
+        <v>5142.97265625</v>
       </c>
       <c r="AA7" s="5" t="n">
-        <v>5768.73984375</v>
+        <v>6078.05859375</v>
       </c>
       <c r="AB7" s="5" t="n">
-        <v>6212.4890625</v>
+        <v>6545.6015625</v>
       </c>
       <c r="AC7" s="5" t="n">
-        <v>6389.98875</v>
+        <v>6732.61875</v>
       </c>
       <c r="AD7" s="5" t="n">
-        <v>6656.23828125</v>
+        <v>7013.14453125</v>
       </c>
       <c r="AE7" s="5" t="n">
-        <v>6656.23828125</v>
+        <v>7013.14453125</v>
       </c>
       <c r="AF7" s="5" t="n">
-        <v>6922.4878125</v>
+        <v>7293.670312499999</v>
       </c>
       <c r="AG7" s="5" t="n">
-        <v>7099.987499999999</v>
+        <v>7480.6875</v>
       </c>
       <c r="AH7" s="5" t="n">
-        <v>7277.4871875</v>
+        <v>7667.7046875</v>
       </c>
       <c r="AI7" s="5" t="n">
-        <v>7543.736718749999</v>
+        <v>7948.23046875</v>
       </c>
       <c r="AJ7" s="5" t="n">
-        <v>7543.736718749999</v>
+        <v>7948.23046875</v>
       </c>
       <c r="AK7" s="5" t="n">
-        <v>7277.4871875</v>
+        <v>7667.7046875</v>
       </c>
       <c r="AL7" s="5" t="n">
-        <v>7721.23640625</v>
+        <v>8135.247656250001</v>
       </c>
       <c r="AM7" s="5" t="n">
-        <v>7809.98625</v>
+        <v>8228.75625</v>
       </c>
       <c r="AN7" s="5" t="n">
-        <v>7987.4859375</v>
+        <v>8415.7734375</v>
       </c>
       <c r="AO7" s="5" t="n">
-        <v>7987.4859375</v>
+        <v>8415.7734375</v>
       </c>
       <c r="AP7" s="39" t="n">
-        <v>118836.04078125</v>
+        <v>125208.00703125</v>
       </c>
       <c r="AS7" s="40" t="inlineStr">
         <is>
@@ -4581,61 +4617,61 @@
         </is>
       </c>
       <c r="AT7" s="5" t="n">
-        <v>5177.074218749999</v>
+        <v>5454.667968749999</v>
       </c>
       <c r="AU7" s="5" t="n">
-        <v>6656.23828125</v>
+        <v>7013.14453125</v>
       </c>
       <c r="AV7" s="5" t="n">
-        <v>8135.40234375</v>
+        <v>8571.62109375</v>
       </c>
       <c r="AW7" s="5" t="n">
-        <v>9614.56640625</v>
+        <v>10130.09765625</v>
       </c>
       <c r="AX7" s="5" t="n">
-        <v>10354.1484375</v>
+        <v>10909.3359375</v>
       </c>
       <c r="AY7" s="5" t="n">
-        <v>10649.98125</v>
+        <v>11221.03125</v>
       </c>
       <c r="AZ7" s="5" t="n">
-        <v>11093.73046875</v>
+        <v>11688.57421875</v>
       </c>
       <c r="BA7" s="5" t="n">
-        <v>11093.73046875</v>
+        <v>11688.57421875</v>
       </c>
       <c r="BB7" s="5" t="n">
-        <v>11537.4796875</v>
+        <v>12156.1171875</v>
       </c>
       <c r="BC7" s="5" t="n">
-        <v>11833.3125</v>
+        <v>12467.8125</v>
       </c>
       <c r="BD7" s="5" t="n">
-        <v>12129.1453125</v>
+        <v>12779.5078125</v>
       </c>
       <c r="BE7" s="5" t="n">
-        <v>12572.89453125</v>
+        <v>13247.05078125</v>
       </c>
       <c r="BF7" s="5" t="n">
-        <v>12572.89453125</v>
+        <v>13247.05078125</v>
       </c>
       <c r="BG7" s="5" t="n">
-        <v>12129.1453125</v>
+        <v>12779.5078125</v>
       </c>
       <c r="BH7" s="5" t="n">
-        <v>12868.72734375</v>
+        <v>13558.74609375</v>
       </c>
       <c r="BI7" s="5" t="n">
-        <v>13016.64375</v>
+        <v>13714.59375</v>
       </c>
       <c r="BJ7" s="5" t="n">
-        <v>13312.4765625</v>
+        <v>14026.2890625</v>
       </c>
       <c r="BK7" s="5" t="n">
-        <v>13312.4765625</v>
+        <v>14026.2890625</v>
       </c>
       <c r="BL7" s="39" t="n">
-        <v>198060.06796875</v>
+        <v>208680.01171875</v>
       </c>
     </row>
     <row r="8">
@@ -5021,61 +5057,61 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>-31.9921875</v>
+        <v>-37.16015624999999</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>-41.1328125</v>
+        <v>-47.77734374999999</v>
       </c>
       <c r="D10" s="5" t="n">
-        <v>-50.2734375</v>
+        <v>-58.39453124999999</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>-59.4140625</v>
+        <v>-69.01171874999999</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>-63.984375</v>
+        <v>-74.32031249999999</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>-65.8125</v>
+        <v>-76.44374999999999</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>-68.5546875</v>
+        <v>-79.62890624999999</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>-68.5546875</v>
+        <v>-79.62890624999999</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>-71.296875</v>
+        <v>-82.81406249999999</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>-73.125</v>
+        <v>-84.93749999999999</v>
       </c>
       <c r="L10" s="5" t="n">
-        <v>-74.953125</v>
+        <v>-87.06093749999999</v>
       </c>
       <c r="M10" s="5" t="n">
-        <v>-77.6953125</v>
+        <v>-90.24609374999999</v>
       </c>
       <c r="N10" s="5" t="n">
-        <v>-77.6953125</v>
+        <v>-90.24609374999999</v>
       </c>
       <c r="O10" s="5" t="n">
-        <v>-74.953125</v>
+        <v>-87.06093749999999</v>
       </c>
       <c r="P10" s="5" t="n">
-        <v>-79.5234375</v>
+        <v>-92.36953124999998</v>
       </c>
       <c r="Q10" s="5" t="n">
-        <v>-80.4375</v>
+        <v>-93.43124999999999</v>
       </c>
       <c r="R10" s="5" t="n">
-        <v>-82.265625</v>
+        <v>-95.55468749999999</v>
       </c>
       <c r="S10" s="5" t="n">
-        <v>-82.265625</v>
+        <v>-95.55468749999999</v>
       </c>
       <c r="T10" s="39" t="n">
-        <v>-1223.9296875</v>
+        <v>-1421.64140625</v>
       </c>
       <c r="W10" s="36" t="inlineStr">
         <is>
@@ -5083,61 +5119,61 @@
         </is>
       </c>
       <c r="X10" s="5" t="n">
-        <v>-95.9765625</v>
+        <v>-111.48046875</v>
       </c>
       <c r="Y10" s="5" t="n">
-        <v>-123.3984375</v>
+        <v>-143.33203125</v>
       </c>
       <c r="Z10" s="5" t="n">
-        <v>-150.8203125</v>
+        <v>-175.18359375</v>
       </c>
       <c r="AA10" s="5" t="n">
-        <v>-178.2421875</v>
+        <v>-207.03515625</v>
       </c>
       <c r="AB10" s="5" t="n">
-        <v>-191.953125</v>
+        <v>-222.9609375</v>
       </c>
       <c r="AC10" s="5" t="n">
-        <v>-197.4375</v>
+        <v>-229.33125</v>
       </c>
       <c r="AD10" s="5" t="n">
-        <v>-205.6640625</v>
+        <v>-238.88671875</v>
       </c>
       <c r="AE10" s="5" t="n">
-        <v>-205.6640625</v>
+        <v>-238.88671875</v>
       </c>
       <c r="AF10" s="5" t="n">
-        <v>-213.890625</v>
+        <v>-248.4421875</v>
       </c>
       <c r="AG10" s="5" t="n">
-        <v>-219.375</v>
+        <v>-254.8125</v>
       </c>
       <c r="AH10" s="5" t="n">
-        <v>-224.859375</v>
+        <v>-261.1828125</v>
       </c>
       <c r="AI10" s="5" t="n">
-        <v>-233.0859375</v>
+        <v>-270.7382812499999</v>
       </c>
       <c r="AJ10" s="5" t="n">
-        <v>-233.0859375</v>
+        <v>-270.7382812499999</v>
       </c>
       <c r="AK10" s="5" t="n">
-        <v>-224.859375</v>
+        <v>-261.1828125</v>
       </c>
       <c r="AL10" s="5" t="n">
-        <v>-238.5703125</v>
+        <v>-277.10859375</v>
       </c>
       <c r="AM10" s="5" t="n">
-        <v>-241.3125</v>
+        <v>-280.29375</v>
       </c>
       <c r="AN10" s="5" t="n">
-        <v>-246.796875</v>
+        <v>-286.6640624999999</v>
       </c>
       <c r="AO10" s="5" t="n">
-        <v>-246.796875</v>
+        <v>-286.6640624999999</v>
       </c>
       <c r="AP10" s="39" t="n">
-        <v>-3671.7890625</v>
+        <v>-4264.924218749999</v>
       </c>
       <c r="AS10" s="36" t="inlineStr">
         <is>
@@ -5145,61 +5181,61 @@
         </is>
       </c>
       <c r="AT10" s="5" t="n">
-        <v>-159.9609375</v>
+        <v>-185.8007812499999</v>
       </c>
       <c r="AU10" s="5" t="n">
-        <v>-205.6640625</v>
+        <v>-238.88671875</v>
       </c>
       <c r="AV10" s="5" t="n">
-        <v>-251.3671875000001</v>
+        <v>-291.97265625</v>
       </c>
       <c r="AW10" s="5" t="n">
-        <v>-297.0703125</v>
+        <v>-345.0585937499999</v>
       </c>
       <c r="AX10" s="5" t="n">
-        <v>-319.921875</v>
+        <v>-371.6015624999999</v>
       </c>
       <c r="AY10" s="5" t="n">
-        <v>-329.0625</v>
+        <v>-382.2187499999999</v>
       </c>
       <c r="AZ10" s="5" t="n">
-        <v>-342.7734375</v>
+        <v>-398.1445312499999</v>
       </c>
       <c r="BA10" s="5" t="n">
-        <v>-342.7734375</v>
+        <v>-398.1445312499999</v>
       </c>
       <c r="BB10" s="5" t="n">
-        <v>-356.484375</v>
+        <v>-414.0703124999999</v>
       </c>
       <c r="BC10" s="5" t="n">
-        <v>-365.625</v>
+        <v>-424.6874999999999</v>
       </c>
       <c r="BD10" s="5" t="n">
-        <v>-374.765625</v>
+        <v>-435.3046874999999</v>
       </c>
       <c r="BE10" s="5" t="n">
-        <v>-388.4765625</v>
+        <v>-451.2304687499999</v>
       </c>
       <c r="BF10" s="5" t="n">
-        <v>-388.4765625</v>
+        <v>-451.2304687499999</v>
       </c>
       <c r="BG10" s="5" t="n">
-        <v>-374.765625</v>
+        <v>-435.3046874999999</v>
       </c>
       <c r="BH10" s="5" t="n">
-        <v>-397.6171875</v>
+        <v>-461.8476562499999</v>
       </c>
       <c r="BI10" s="5" t="n">
-        <v>-402.1875</v>
+        <v>-467.1562499999999</v>
       </c>
       <c r="BJ10" s="5" t="n">
-        <v>-411.328125</v>
+        <v>-477.7734374999999</v>
       </c>
       <c r="BK10" s="5" t="n">
-        <v>-411.328125</v>
+        <v>-477.7734374999999</v>
       </c>
       <c r="BL10" s="39" t="n">
-        <v>-6119.6484375</v>
+        <v>-7108.207031249999</v>
       </c>
     </row>
     <row r="11">
@@ -5397,61 +5433,61 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>-3295.337430893333</v>
+        <v>-3300.505399643333</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>-3304.478055893333</v>
+        <v>-3311.122587143333</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>-3313.618680893333</v>
+        <v>-3321.739774643333</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>-3322.759305893333</v>
+        <v>-3332.356962143333</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>-3327.329618393333</v>
+        <v>-3337.665555893333</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>-3329.157743393333</v>
+        <v>-3339.788993393333</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>-3411.899930893333</v>
+        <v>-3422.974149643333</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>-3411.899930893333</v>
+        <v>-3422.974149643333</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>-3414.642118393333</v>
+        <v>-3426.159305893333</v>
       </c>
       <c r="K12" s="5" t="n">
-        <v>-3416.470243393333</v>
+        <v>-3428.282743393333</v>
       </c>
       <c r="L12" s="5" t="n">
-        <v>-3418.298368393333</v>
+        <v>-3430.406180893333</v>
       </c>
       <c r="M12" s="5" t="n">
-        <v>-3421.040555893333</v>
+        <v>-3433.591337143333</v>
       </c>
       <c r="N12" s="5" t="n">
-        <v>-3581.040555893333</v>
+        <v>-3593.591337143333</v>
       </c>
       <c r="O12" s="5" t="n">
-        <v>-3578.298368393333</v>
+        <v>-3590.406180893333</v>
       </c>
       <c r="P12" s="5" t="n">
-        <v>-3582.868680893333</v>
+        <v>-3595.714774643333</v>
       </c>
       <c r="Q12" s="5" t="n">
-        <v>-3583.782743393333</v>
+        <v>-3596.776493393334</v>
       </c>
       <c r="R12" s="5" t="n">
-        <v>-3585.610868393333</v>
+        <v>-3598.899930893333</v>
       </c>
       <c r="S12" s="5" t="n">
-        <v>-3585.610868393333</v>
+        <v>-3598.899930893333</v>
       </c>
       <c r="T12" s="39" t="n">
-        <v>-61884.14406858001</v>
+        <v>-62081.85578733001</v>
       </c>
       <c r="W12" s="40" t="inlineStr">
         <is>
@@ -5459,61 +5495,61 @@
         </is>
       </c>
       <c r="X12" s="5" t="n">
-        <v>-6866.01229268</v>
+        <v>-6881.51619893</v>
       </c>
       <c r="Y12" s="5" t="n">
-        <v>-6893.43416768</v>
+        <v>-6913.36776143</v>
       </c>
       <c r="Z12" s="5" t="n">
-        <v>-6920.85604268</v>
+        <v>-6945.21932393</v>
       </c>
       <c r="AA12" s="5" t="n">
-        <v>-6948.27791768</v>
+        <v>-6977.07088643</v>
       </c>
       <c r="AB12" s="5" t="n">
-        <v>-6961.98885518</v>
+        <v>-6992.99666768</v>
       </c>
       <c r="AC12" s="5" t="n">
-        <v>-6967.47323018</v>
+        <v>-6999.36698018</v>
       </c>
       <c r="AD12" s="5" t="n">
-        <v>-7055.69979268</v>
+        <v>-7088.92244893</v>
       </c>
       <c r="AE12" s="5" t="n">
-        <v>-7055.69979268</v>
+        <v>-7088.92244893</v>
       </c>
       <c r="AF12" s="5" t="n">
-        <v>-7063.92635518</v>
+        <v>-7098.477917679999</v>
       </c>
       <c r="AG12" s="5" t="n">
-        <v>-7069.41073018</v>
+        <v>-7104.84823018</v>
       </c>
       <c r="AH12" s="5" t="n">
-        <v>-7074.89510518</v>
+        <v>-7111.21854268</v>
       </c>
       <c r="AI12" s="5" t="n">
-        <v>-7083.12166768</v>
+        <v>-7120.77401143</v>
       </c>
       <c r="AJ12" s="5" t="n">
-        <v>-7243.12166768</v>
+        <v>-7280.77401143</v>
       </c>
       <c r="AK12" s="5" t="n">
-        <v>-7234.89510518</v>
+        <v>-7271.21854268</v>
       </c>
       <c r="AL12" s="5" t="n">
-        <v>-7248.60604268</v>
+        <v>-7287.14432393</v>
       </c>
       <c r="AM12" s="5" t="n">
-        <v>-7251.34823018</v>
+        <v>-7290.329480179999</v>
       </c>
       <c r="AN12" s="5" t="n">
-        <v>-7256.83260518</v>
+        <v>-7296.69979268</v>
       </c>
       <c r="AO12" s="5" t="n">
-        <v>-7256.83260518</v>
+        <v>-7296.69979268</v>
       </c>
       <c r="AP12" s="39" t="n">
-        <v>-127452.4322057399</v>
+        <v>-128045.56736199</v>
       </c>
       <c r="AS12" s="40" t="inlineStr">
         <is>
@@ -5521,249 +5557,249 @@
         </is>
       </c>
       <c r="AT12" s="5" t="n">
-        <v>-10436.68715446667</v>
+        <v>-10462.52699821667</v>
       </c>
       <c r="AU12" s="5" t="n">
-        <v>-10482.39027946667</v>
+        <v>-10515.61293571667</v>
       </c>
       <c r="AV12" s="5" t="n">
-        <v>-10528.09340446667</v>
+        <v>-10568.69887321667</v>
       </c>
       <c r="AW12" s="5" t="n">
-        <v>-10573.79652946667</v>
+        <v>-10621.78481071667</v>
       </c>
       <c r="AX12" s="5" t="n">
-        <v>-10596.64809196667</v>
+        <v>-10648.32777946667</v>
       </c>
       <c r="AY12" s="5" t="n">
-        <v>-10605.78871696667</v>
+        <v>-10658.94496696667</v>
       </c>
       <c r="AZ12" s="5" t="n">
-        <v>-10699.49965446667</v>
+        <v>-10754.87074821667</v>
       </c>
       <c r="BA12" s="5" t="n">
-        <v>-10699.49965446667</v>
+        <v>-10754.87074821667</v>
       </c>
       <c r="BB12" s="5" t="n">
-        <v>-10713.21059196667</v>
+        <v>-10770.79652946667</v>
       </c>
       <c r="BC12" s="5" t="n">
-        <v>-10722.35121696667</v>
+        <v>-10781.41371696667</v>
       </c>
       <c r="BD12" s="5" t="n">
-        <v>-10731.49184196667</v>
+        <v>-10792.03090446667</v>
       </c>
       <c r="BE12" s="5" t="n">
-        <v>-10745.20277946667</v>
+        <v>-10807.95668571667</v>
       </c>
       <c r="BF12" s="5" t="n">
-        <v>-10905.20277946667</v>
+        <v>-10967.95668571667</v>
       </c>
       <c r="BG12" s="5" t="n">
-        <v>-10891.49184196667</v>
+        <v>-10952.03090446667</v>
       </c>
       <c r="BH12" s="5" t="n">
-        <v>-10914.34340446667</v>
+        <v>-10978.57387321667</v>
       </c>
       <c r="BI12" s="5" t="n">
-        <v>-10918.91371696667</v>
+        <v>-10983.88246696667</v>
       </c>
       <c r="BJ12" s="5" t="n">
-        <v>-10928.05434196667</v>
+        <v>-10994.49965446667</v>
       </c>
       <c r="BK12" s="5" t="n">
-        <v>-10928.05434196667</v>
+        <v>-10994.49965446667</v>
       </c>
       <c r="BL12" s="39" t="n">
-        <v>-193020.7203429</v>
+        <v>-194009.27893665</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="40" t="inlineStr">
         <is>
-          <t>EBITDA / BENEFICIO NETO</t>
+          <t>EBITDA</t>
         </is>
       </c>
       <c r="B13" s="41" t="n">
-        <v>-2259.922587143334</v>
+        <v>-2209.571805893333</v>
       </c>
       <c r="C13" s="41" t="n">
-        <v>-1973.230399643333</v>
+        <v>-1908.493680893333</v>
       </c>
       <c r="D13" s="41" t="n">
-        <v>-1686.538212143334</v>
+        <v>-1607.415555893333</v>
       </c>
       <c r="E13" s="41" t="n">
-        <v>-1399.846024643334</v>
+        <v>-1306.337430893333</v>
       </c>
       <c r="F13" s="41" t="n">
-        <v>-1256.499930893333</v>
+        <v>-1155.798368393333</v>
       </c>
       <c r="G13" s="41" t="n">
-        <v>-1199.161493393333</v>
+        <v>-1095.582743393333</v>
       </c>
       <c r="H13" s="41" t="n">
-        <v>-1193.153837143333</v>
+        <v>-1085.259305893333</v>
       </c>
       <c r="I13" s="41" t="n">
-        <v>-1193.153837143333</v>
+        <v>-1085.259305893333</v>
       </c>
       <c r="J13" s="41" t="n">
-        <v>-1107.146180893334</v>
+        <v>-994.9358683933328</v>
       </c>
       <c r="K13" s="41" t="n">
-        <v>-1049.807743393334</v>
+        <v>-934.7202433933335</v>
       </c>
       <c r="L13" s="41" t="n">
-        <v>-992.4693058933335</v>
+        <v>-874.5046183933327</v>
       </c>
       <c r="M13" s="41" t="n">
-        <v>-906.4616496433337</v>
+        <v>-784.1811808933335</v>
       </c>
       <c r="N13" s="41" t="n">
-        <v>-1066.461649643334</v>
+        <v>-944.1811808933335</v>
       </c>
       <c r="O13" s="41" t="n">
-        <v>-1152.469305893334</v>
+        <v>-1034.504618393333</v>
       </c>
       <c r="P13" s="41" t="n">
-        <v>-1009.123212143333</v>
+        <v>-883.9655558933332</v>
       </c>
       <c r="Q13" s="41" t="n">
-        <v>-980.4539933933338</v>
+        <v>-853.8577433933333</v>
       </c>
       <c r="R13" s="41" t="n">
-        <v>-923.1155558933333</v>
+        <v>-793.6421183933335</v>
       </c>
       <c r="S13" s="41" t="n">
-        <v>-923.1155558933333</v>
+        <v>-793.6421183933335</v>
       </c>
       <c r="T13" s="39" t="n">
-        <v>-22272.13047483</v>
+        <v>-20345.85344358</v>
       </c>
       <c r="W13" s="40" t="inlineStr">
         <is>
-          <t>EBITDA / BENEFICIO NETO</t>
+          <t>EBITDA</t>
         </is>
       </c>
       <c r="X13" s="41" t="n">
-        <v>-3759.76776143</v>
+        <v>-3608.71541768</v>
       </c>
       <c r="Y13" s="41" t="n">
-        <v>-2899.69119893</v>
+        <v>-2705.48104268</v>
       </c>
       <c r="Z13" s="41" t="n">
-        <v>-2039.614636429999</v>
+        <v>-1802.24666768</v>
       </c>
       <c r="AA13" s="41" t="n">
-        <v>-1179.53807393</v>
+        <v>-899.0122926799995</v>
       </c>
       <c r="AB13" s="41" t="n">
-        <v>-749.4997926799997</v>
+        <v>-447.3951051799995</v>
       </c>
       <c r="AC13" s="41" t="n">
-        <v>-577.4844801799991</v>
+        <v>-266.7482301800001</v>
       </c>
       <c r="AD13" s="41" t="n">
-        <v>-399.4615114299995</v>
+        <v>-75.77791767999952</v>
       </c>
       <c r="AE13" s="41" t="n">
-        <v>-399.4615114299995</v>
-      </c>
-      <c r="AF13" s="41" t="n">
-        <v>-141.43854268</v>
+        <v>-75.77791767999952</v>
+      </c>
+      <c r="AF13" s="42" t="n">
+        <v>195.1923948200001</v>
       </c>
       <c r="AG13" s="42" t="n">
-        <v>30.57676981999975</v>
+        <v>375.8392698200005</v>
       </c>
       <c r="AH13" s="42" t="n">
-        <v>202.5920823200004</v>
+        <v>556.4861448199999</v>
       </c>
       <c r="AI13" s="42" t="n">
-        <v>460.6150510699999</v>
+        <v>827.4564573200005</v>
       </c>
       <c r="AJ13" s="42" t="n">
-        <v>300.6150510699999</v>
+        <v>667.4564573200005</v>
       </c>
       <c r="AK13" s="42" t="n">
-        <v>42.59208232000037</v>
+        <v>396.4861448199999</v>
       </c>
       <c r="AL13" s="42" t="n">
-        <v>472.6303635700006</v>
+        <v>848.1033323200008</v>
       </c>
       <c r="AM13" s="42" t="n">
-        <v>558.6380198200004</v>
+        <v>938.426769820001</v>
       </c>
       <c r="AN13" s="42" t="n">
-        <v>730.6533323200001</v>
+        <v>1119.07364482</v>
       </c>
       <c r="AO13" s="42" t="n">
-        <v>730.6533323200001</v>
+        <v>1119.07364482</v>
       </c>
       <c r="AP13" s="39" t="n">
-        <v>-8616.391424490001</v>
+        <v>-2837.560330739992</v>
       </c>
       <c r="AS13" s="40" t="inlineStr">
         <is>
-          <t>EBITDA / BENEFICIO NETO</t>
+          <t>EBITDA</t>
         </is>
       </c>
       <c r="AT13" s="41" t="n">
-        <v>-5259.612935716667</v>
+        <v>-5007.859029466667</v>
       </c>
       <c r="AU13" s="41" t="n">
-        <v>-3826.151998216666</v>
+        <v>-3502.468404466666</v>
       </c>
       <c r="AV13" s="41" t="n">
-        <v>-2392.691060716666</v>
+        <v>-1997.077779466666</v>
       </c>
       <c r="AW13" s="41" t="n">
-        <v>-959.2301232166665</v>
-      </c>
-      <c r="AX13" s="41" t="n">
-        <v>-242.4996544666683</v>
+        <v>-491.6871544666665</v>
+      </c>
+      <c r="AX13" s="42" t="n">
+        <v>261.0081580333317</v>
       </c>
       <c r="AY13" s="42" t="n">
-        <v>44.19253303333426</v>
+        <v>562.0862830333335</v>
       </c>
       <c r="AZ13" s="42" t="n">
-        <v>394.2308142833335</v>
+        <v>933.7034705333335</v>
       </c>
       <c r="BA13" s="42" t="n">
-        <v>394.2308142833335</v>
+        <v>933.7034705333335</v>
       </c>
       <c r="BB13" s="42" t="n">
-        <v>824.2690955333328</v>
+        <v>1385.320658033334</v>
       </c>
       <c r="BC13" s="42" t="n">
-        <v>1110.961283033334</v>
+        <v>1686.398783033334</v>
       </c>
       <c r="BD13" s="42" t="n">
-        <v>1397.653470533334</v>
+        <v>1987.476908033334</v>
       </c>
       <c r="BE13" s="42" t="n">
-        <v>1827.691751783334</v>
+        <v>2439.094095533334</v>
       </c>
       <c r="BF13" s="42" t="n">
-        <v>1667.691751783334</v>
+        <v>2279.094095533334</v>
       </c>
       <c r="BG13" s="42" t="n">
-        <v>1237.653470533334</v>
+        <v>1827.476908033334</v>
       </c>
       <c r="BH13" s="42" t="n">
-        <v>1954.383939283334</v>
+        <v>2580.172220533334</v>
       </c>
       <c r="BI13" s="42" t="n">
-        <v>2097.730033033333</v>
+        <v>2730.711283033334</v>
       </c>
       <c r="BJ13" s="42" t="n">
-        <v>2384.422220533334</v>
+        <v>3031.789408033334</v>
       </c>
       <c r="BK13" s="42" t="n">
-        <v>2384.422220533334</v>
+        <v>3031.789408033334</v>
       </c>
       <c r="BL13" s="39" t="n">
-        <v>5039.347625850003</v>
+        <v>14670.7327821</v>
       </c>
     </row>
     <row r="14">
@@ -5773,61 +5809,61 @@
         </is>
       </c>
       <c r="B14" s="8" t="n">
-        <v>-2.182625254780479</v>
+        <v>-2.025395329790974</v>
       </c>
       <c r="C14" s="8" t="n">
-        <v>-1.48224140743409</v>
+        <v>-1.36065474794455</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>-1.036542595486388</v>
+        <v>-0.9376380140422802</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>-0.7279818795225941</v>
+        <v>-0.6447802751868627</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>-0.6067615982511035</v>
+        <v>-0.5297290206365201</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>-0.5629876077919542</v>
+        <v>-0.4881827342711182</v>
       </c>
       <c r="H14" s="8" t="n">
-        <v>-0.5377604226568944</v>
+        <v>-0.4642393869358488</v>
       </c>
       <c r="I14" s="8" t="n">
-        <v>-0.5377604226568944</v>
+        <v>-0.4642393869358488</v>
       </c>
       <c r="J14" s="8" t="n">
-        <v>-0.4798041733901574</v>
+        <v>-0.4092325917260876</v>
       </c>
       <c r="K14" s="8" t="n">
-        <v>-0.4435815175984466</v>
+        <v>-0.3748533447199874</v>
       </c>
       <c r="L14" s="8" t="n">
-        <v>-0.4091258206258437</v>
+        <v>-0.3421511341532085</v>
       </c>
       <c r="M14" s="8" t="n">
-        <v>-0.3604824837233456</v>
+        <v>-0.2959833074706979</v>
       </c>
       <c r="N14" s="8" t="n">
-        <v>-0.4241114275605499</v>
+        <v>-0.356374107899449</v>
       </c>
       <c r="O14" s="8" t="n">
-        <v>-0.4750826526522141</v>
+        <v>-0.4047513541098409</v>
       </c>
       <c r="P14" s="8" t="n">
-        <v>-0.3920835313343699</v>
+        <v>-0.3259761447634171</v>
       </c>
       <c r="Q14" s="8" t="n">
-        <v>-0.3766155132705902</v>
+        <v>-0.3112953102943108</v>
       </c>
       <c r="R14" s="8" t="n">
-        <v>-0.3467106783472819</v>
+        <v>-0.2829123636540388</v>
       </c>
       <c r="S14" s="8" t="n">
-        <v>-0.3467106783472819</v>
+        <v>-0.2829123636540388</v>
       </c>
       <c r="T14" s="43" t="n">
-        <v>-0.3467106783472819</v>
+        <v>-0.2829123636540388</v>
       </c>
       <c r="W14" s="36" t="inlineStr">
         <is>
@@ -5835,61 +5871,61 @@
         </is>
       </c>
       <c r="X14" s="8" t="n">
-        <v>-1.210390142696529</v>
+        <v>-1.102638278001664</v>
       </c>
       <c r="Y14" s="8" t="n">
-        <v>-0.7260585424799065</v>
+        <v>-0.6429548187750864</v>
       </c>
       <c r="Z14" s="8" t="n">
-        <v>-0.4178475241602376</v>
+        <v>-0.3504289810854465</v>
       </c>
       <c r="AA14" s="8" t="n">
-        <v>-0.204470665323544</v>
+        <v>-0.1479110934541572</v>
       </c>
       <c r="AB14" s="8" t="n">
-        <v>-0.1206440422091286</v>
+        <v>-0.068350494741865</v>
       </c>
       <c r="AC14" s="8" t="n">
-        <v>-0.09037331719558959</v>
+        <v>-0.039620278540204</v>
       </c>
       <c r="AD14" s="8" t="n">
-        <v>-0.06001310267921826</v>
+        <v>-0.01080512704997584</v>
       </c>
       <c r="AE14" s="8" t="n">
-        <v>-0.06001310267921826</v>
+        <v>-0.01080512704997584</v>
       </c>
       <c r="AF14" s="8" t="n">
-        <v>-0.02043175033469948</v>
+        <v>0.02676188893340525</v>
       </c>
       <c r="AG14" s="8" t="n">
-        <v>0.004306594880624756</v>
+        <v>0.0502412739230185</v>
       </c>
       <c r="AH14" s="8" t="n">
-        <v>0.02783819154886013</v>
+        <v>0.07257532305947978</v>
       </c>
       <c r="AI14" s="8" t="n">
-        <v>0.06105926919813343</v>
+        <v>0.1041057453697782</v>
       </c>
       <c r="AJ14" s="8" t="n">
-        <v>0.03984962125239864</v>
+        <v>0.08397547856019452</v>
       </c>
       <c r="AK14" s="8" t="n">
-        <v>0.005852580873403341</v>
+        <v>0.05170858307393571</v>
       </c>
       <c r="AL14" s="8" t="n">
-        <v>0.06121174624149924</v>
+        <v>0.1042504626971541</v>
       </c>
       <c r="AM14" s="8" t="n">
-        <v>0.07152868160555345</v>
+        <v>0.1140423584451175</v>
       </c>
       <c r="AN14" s="8" t="n">
-        <v>0.09147475664272493</v>
+        <v>0.13297335689118</v>
       </c>
       <c r="AO14" s="8" t="n">
-        <v>0.09147475664272493</v>
+        <v>0.13297335689118</v>
       </c>
       <c r="AP14" s="43" t="n">
-        <v>0.09147475664272493</v>
+        <v>0.13297335689118</v>
       </c>
       <c r="AS14" s="36" t="inlineStr">
         <is>
@@ -5897,249 +5933,249 @@
         </is>
       </c>
       <c r="AT14" s="8" t="n">
-        <v>-1.015943120279739</v>
+        <v>-0.9180868676438021</v>
       </c>
       <c r="AU14" s="8" t="n">
-        <v>-0.5748219694890699</v>
+        <v>-0.4994148329411939</v>
       </c>
       <c r="AV14" s="8" t="n">
-        <v>-0.2941085098950078</v>
+        <v>-0.2329871744940798</v>
       </c>
       <c r="AW14" s="8" t="n">
-        <v>-0.09976842248373403</v>
+        <v>-0.04853725710761619</v>
       </c>
       <c r="AX14" s="8" t="n">
-        <v>-0.02342053100073381</v>
+        <v>0.02392521043706577</v>
       </c>
       <c r="AY14" s="8" t="n">
-        <v>0.004149540923683246</v>
+        <v>0.05009221260597893</v>
       </c>
       <c r="AZ14" s="8" t="n">
-        <v>0.03553636131631689</v>
+        <v>0.07988172492719867</v>
       </c>
       <c r="BA14" s="8" t="n">
-        <v>0.03553636131631689</v>
+        <v>0.07988172492719867</v>
       </c>
       <c r="BB14" s="8" t="n">
-        <v>0.07144273427639201</v>
+        <v>0.1139607850653039</v>
       </c>
       <c r="BC14" s="8" t="n">
-        <v>0.09388421737643907</v>
+        <v>0.1352601976516196</v>
       </c>
       <c r="BD14" s="8" t="n">
-        <v>0.1152309939838009</v>
+        <v>0.1555206145020175</v>
       </c>
       <c r="BE14" s="8" t="n">
-        <v>0.1453676197824292</v>
+        <v>0.1841235559378734</v>
       </c>
       <c r="BF14" s="8" t="n">
-        <v>0.1326418310149883</v>
+        <v>0.1720453958521231</v>
       </c>
       <c r="BG14" s="8" t="n">
-        <v>0.1020396275785268</v>
+        <v>0.1430005705106911</v>
       </c>
       <c r="BH14" s="8" t="n">
-        <v>0.1518708017566731</v>
+        <v>0.1902957841892682</v>
       </c>
       <c r="BI14" s="8" t="n">
-        <v>0.161157520580782</v>
+        <v>0.1991098921930031</v>
       </c>
       <c r="BJ14" s="8" t="n">
-        <v>0.1791118436407263</v>
+        <v>0.2161505010002237</v>
       </c>
       <c r="BK14" s="8" t="n">
-        <v>0.1791118436407263</v>
+        <v>0.2161505010002237</v>
       </c>
       <c r="BL14" s="43" t="n">
-        <v>0.1791118436407263</v>
+        <v>0.2161505010002237</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="36" t="inlineStr">
         <is>
-          <t>Break-even (h/mes necesarias)</t>
+          <t>Break-even mensual (h/mes)</t>
         </is>
       </c>
       <c r="B15" s="37" t="n">
-        <v>455.3293209701876</v>
+        <v>152.4215433626032</v>
       </c>
       <c r="C15" s="37" t="n">
-        <v>455.3293209701876</v>
+        <v>152.4215433626032</v>
       </c>
       <c r="D15" s="37" t="n">
-        <v>455.3293209701876</v>
+        <v>152.4215433626032</v>
       </c>
       <c r="E15" s="37" t="n">
-        <v>455.3293209701876</v>
+        <v>152.4215433626032</v>
       </c>
       <c r="F15" s="37" t="n">
-        <v>455.3293209701876</v>
+        <v>152.4215433626032</v>
       </c>
       <c r="G15" s="37" t="n">
-        <v>455.3293209701876</v>
+        <v>152.4215433626032</v>
       </c>
       <c r="H15" s="37" t="n">
-        <v>466.4915924924424</v>
+        <v>156.1581150580726</v>
       </c>
       <c r="I15" s="37" t="n">
-        <v>466.4915924924424</v>
+        <v>156.1581150580726</v>
       </c>
       <c r="J15" s="37" t="n">
-        <v>466.4915924924424</v>
+        <v>156.1581150580726</v>
       </c>
       <c r="K15" s="37" t="n">
-        <v>466.4915924924424</v>
+        <v>156.1581150580726</v>
       </c>
       <c r="L15" s="37" t="n">
-        <v>466.4915924924424</v>
+        <v>156.1581150580726</v>
       </c>
       <c r="M15" s="37" t="n">
-        <v>466.4915924924424</v>
+        <v>156.1581150580726</v>
       </c>
       <c r="N15" s="37" t="n">
-        <v>488.8161355369519</v>
+        <v>163.6312584490114</v>
       </c>
       <c r="O15" s="37" t="n">
-        <v>488.8161355369519</v>
+        <v>163.6312584490114</v>
       </c>
       <c r="P15" s="37" t="n">
-        <v>488.8161355369519</v>
+        <v>163.6312584490114</v>
       </c>
       <c r="Q15" s="37" t="n">
-        <v>488.8161355369519</v>
+        <v>163.6312584490114</v>
       </c>
       <c r="R15" s="37" t="n">
-        <v>488.8161355369519</v>
+        <v>163.6312584490114</v>
       </c>
       <c r="S15" s="37" t="n">
-        <v>488.8161355369519</v>
+        <v>163.6312584490114</v>
       </c>
       <c r="T15" s="38" t="n">
-        <v>488.8161355369519</v>
+        <v>163.6312584490114</v>
       </c>
       <c r="W15" s="36" t="inlineStr">
         <is>
-          <t>Break-even (h/mes necesarias)</t>
+          <t>Break-even mensual (h/mes)</t>
         </is>
       </c>
       <c r="X15" s="37" t="n">
-        <v>944.6122129454446</v>
+        <v>316.2090485838393</v>
       </c>
       <c r="Y15" s="37" t="n">
-        <v>944.6122129454446</v>
+        <v>316.2090485838393</v>
       </c>
       <c r="Z15" s="37" t="n">
-        <v>944.6122129454446</v>
+        <v>316.2090485838393</v>
       </c>
       <c r="AA15" s="37" t="n">
-        <v>944.6122129454446</v>
+        <v>316.2090485838393</v>
       </c>
       <c r="AB15" s="37" t="n">
-        <v>944.6122129454446</v>
+        <v>316.2090485838393</v>
       </c>
       <c r="AC15" s="37" t="n">
-        <v>944.6122129454446</v>
+        <v>316.2090485838393</v>
       </c>
       <c r="AD15" s="37" t="n">
-        <v>955.7744844676994</v>
+        <v>319.9456202793087</v>
       </c>
       <c r="AE15" s="37" t="n">
-        <v>955.7744844676994</v>
+        <v>319.9456202793087</v>
       </c>
       <c r="AF15" s="37" t="n">
-        <v>955.7744844676994</v>
+        <v>319.9456202793087</v>
       </c>
       <c r="AG15" s="37" t="n">
-        <v>955.7744844676994</v>
+        <v>319.9456202793087</v>
       </c>
       <c r="AH15" s="37" t="n">
-        <v>955.7744844676994</v>
+        <v>319.9456202793087</v>
       </c>
       <c r="AI15" s="37" t="n">
-        <v>955.7744844676994</v>
+        <v>319.9456202793087</v>
       </c>
       <c r="AJ15" s="37" t="n">
-        <v>978.099027512209</v>
+        <v>327.4187636702475</v>
       </c>
       <c r="AK15" s="37" t="n">
-        <v>978.099027512209</v>
+        <v>327.4187636702475</v>
       </c>
       <c r="AL15" s="37" t="n">
-        <v>978.099027512209</v>
+        <v>327.4187636702475</v>
       </c>
       <c r="AM15" s="37" t="n">
-        <v>978.099027512209</v>
+        <v>327.4187636702475</v>
       </c>
       <c r="AN15" s="37" t="n">
-        <v>978.099027512209</v>
+        <v>327.4187636702475</v>
       </c>
       <c r="AO15" s="37" t="n">
-        <v>978.099027512209</v>
+        <v>327.4187636702475</v>
       </c>
       <c r="AP15" s="38" t="n">
-        <v>978.099027512209</v>
+        <v>327.4187636702475</v>
       </c>
       <c r="AS15" s="36" t="inlineStr">
         <is>
-          <t>Break-even (h/mes necesarias)</t>
+          <t>Break-even mensual (h/mes)</t>
         </is>
       </c>
       <c r="AT15" s="37" t="n">
-        <v>1433.895104920702</v>
+        <v>479.9965538050755</v>
       </c>
       <c r="AU15" s="37" t="n">
-        <v>1433.895104920702</v>
+        <v>479.9965538050755</v>
       </c>
       <c r="AV15" s="37" t="n">
-        <v>1433.895104920702</v>
+        <v>479.9965538050755</v>
       </c>
       <c r="AW15" s="37" t="n">
-        <v>1433.895104920702</v>
+        <v>479.9965538050755</v>
       </c>
       <c r="AX15" s="37" t="n">
-        <v>1433.895104920702</v>
+        <v>479.9965538050755</v>
       </c>
       <c r="AY15" s="37" t="n">
-        <v>1433.895104920702</v>
+        <v>479.9965538050755</v>
       </c>
       <c r="AZ15" s="37" t="n">
-        <v>1445.057376442956</v>
+        <v>483.7331255005449</v>
       </c>
       <c r="BA15" s="37" t="n">
-        <v>1445.057376442956</v>
+        <v>483.7331255005449</v>
       </c>
       <c r="BB15" s="37" t="n">
-        <v>1445.057376442956</v>
+        <v>483.7331255005449</v>
       </c>
       <c r="BC15" s="37" t="n">
-        <v>1445.057376442956</v>
+        <v>483.7331255005449</v>
       </c>
       <c r="BD15" s="37" t="n">
-        <v>1445.057376442956</v>
+        <v>483.7331255005449</v>
       </c>
       <c r="BE15" s="37" t="n">
-        <v>1445.057376442956</v>
+        <v>483.7331255005449</v>
       </c>
       <c r="BF15" s="37" t="n">
-        <v>1467.381919487466</v>
+        <v>491.2062688914837</v>
       </c>
       <c r="BG15" s="37" t="n">
-        <v>1467.381919487466</v>
+        <v>491.2062688914837</v>
       </c>
       <c r="BH15" s="37" t="n">
-        <v>1467.381919487466</v>
+        <v>491.2062688914837</v>
       </c>
       <c r="BI15" s="37" t="n">
-        <v>1467.381919487466</v>
+        <v>491.2062688914837</v>
       </c>
       <c r="BJ15" s="37" t="n">
-        <v>1467.381919487466</v>
+        <v>491.2062688914837</v>
       </c>
       <c r="BK15" s="37" t="n">
-        <v>1467.381919487466</v>
+        <v>491.2062688914837</v>
       </c>
       <c r="BL15" s="38" t="n">
-        <v>1467.381919487466</v>
+        <v>491.2062688914837</v>
       </c>
     </row>
   </sheetData>
@@ -6150,4 +6186,1489 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:U36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="10" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>ESCENARIO A – ESTRUCTURA COMPLETA (oficina + vehículo leasing)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>INVERSIÓN INICIAL (setup)</t>
+        </is>
+      </c>
+      <c r="B3" s="44" t="n">
+        <v>-2800</v>
+      </c>
+      <c r="C3" s="45" t="inlineStr"/>
+      <c r="D3" s="45" t="inlineStr"/>
+      <c r="E3" s="45" t="inlineStr"/>
+      <c r="F3" s="45" t="inlineStr"/>
+      <c r="G3" s="45" t="inlineStr"/>
+      <c r="H3" s="45" t="inlineStr"/>
+      <c r="I3" s="45" t="inlineStr"/>
+      <c r="J3" s="45" t="inlineStr"/>
+      <c r="K3" s="45" t="inlineStr"/>
+      <c r="L3" s="45" t="inlineStr"/>
+      <c r="M3" s="45" t="inlineStr"/>
+      <c r="N3" s="45" t="inlineStr"/>
+      <c r="O3" s="45" t="inlineStr"/>
+      <c r="P3" s="45" t="inlineStr"/>
+      <c r="Q3" s="45" t="inlineStr"/>
+      <c r="R3" s="45" t="inlineStr"/>
+      <c r="S3" s="45" t="inlineStr"/>
+      <c r="T3" s="45" t="inlineStr"/>
+      <c r="U3" s="45" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="46" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="B4" s="33" t="inlineStr">
+        <is>
+          <t>Jul'26</t>
+        </is>
+      </c>
+      <c r="C4" s="33" t="inlineStr">
+        <is>
+          <t>Ago'26</t>
+        </is>
+      </c>
+      <c r="D4" s="33" t="inlineStr">
+        <is>
+          <t>Sep'26</t>
+        </is>
+      </c>
+      <c r="E4" s="33" t="inlineStr">
+        <is>
+          <t>Oct'26</t>
+        </is>
+      </c>
+      <c r="F4" s="33" t="inlineStr">
+        <is>
+          <t>Nov'26</t>
+        </is>
+      </c>
+      <c r="G4" s="33" t="inlineStr">
+        <is>
+          <t>Dic'26</t>
+        </is>
+      </c>
+      <c r="H4" s="33" t="inlineStr">
+        <is>
+          <t>Ene'27</t>
+        </is>
+      </c>
+      <c r="I4" s="33" t="inlineStr">
+        <is>
+          <t>Feb'27</t>
+        </is>
+      </c>
+      <c r="J4" s="33" t="inlineStr">
+        <is>
+          <t>Mar'27</t>
+        </is>
+      </c>
+      <c r="K4" s="33" t="inlineStr">
+        <is>
+          <t>Abr'27</t>
+        </is>
+      </c>
+      <c r="L4" s="33" t="inlineStr">
+        <is>
+          <t>May'27</t>
+        </is>
+      </c>
+      <c r="M4" s="33" t="inlineStr">
+        <is>
+          <t>Jun'27</t>
+        </is>
+      </c>
+      <c r="N4" s="33" t="inlineStr">
+        <is>
+          <t>Jul'27</t>
+        </is>
+      </c>
+      <c r="O4" s="33" t="inlineStr">
+        <is>
+          <t>Ago'27</t>
+        </is>
+      </c>
+      <c r="P4" s="33" t="inlineStr">
+        <is>
+          <t>Sep'27</t>
+        </is>
+      </c>
+      <c r="Q4" s="33" t="inlineStr">
+        <is>
+          <t>Oct'27</t>
+        </is>
+      </c>
+      <c r="R4" s="33" t="inlineStr">
+        <is>
+          <t>Nov'27</t>
+        </is>
+      </c>
+      <c r="S4" s="33" t="inlineStr">
+        <is>
+          <t>Dic'27</t>
+        </is>
+      </c>
+      <c r="U4" s="47" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="36" t="inlineStr">
+        <is>
+          <t>Nº empleados activos</t>
+        </is>
+      </c>
+      <c r="B5" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" s="48" t="n">
+        <v>2</v>
+      </c>
+      <c r="I5" s="48" t="n">
+        <v>2</v>
+      </c>
+      <c r="J5" s="48" t="n">
+        <v>2</v>
+      </c>
+      <c r="K5" s="48" t="n">
+        <v>2</v>
+      </c>
+      <c r="L5" s="48" t="n">
+        <v>2</v>
+      </c>
+      <c r="M5" s="48" t="n">
+        <v>3</v>
+      </c>
+      <c r="N5" s="48" t="n">
+        <v>3</v>
+      </c>
+      <c r="O5" s="48" t="n">
+        <v>3</v>
+      </c>
+      <c r="P5" s="48" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q5" s="48" t="n">
+        <v>3</v>
+      </c>
+      <c r="R5" s="48" t="n">
+        <v>3</v>
+      </c>
+      <c r="S5" s="48" t="n">
+        <v>3</v>
+      </c>
+      <c r="U5" s="49" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="36" t="inlineStr">
+        <is>
+          <t>Horas facturadas/mes</t>
+        </is>
+      </c>
+      <c r="B6" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="37" t="n">
+        <v>60.46875</v>
+      </c>
+      <c r="E6" s="37" t="n">
+        <v>90</v>
+      </c>
+      <c r="F6" s="37" t="n">
+        <v>109.6875</v>
+      </c>
+      <c r="G6" s="37" t="n">
+        <v>125.15625</v>
+      </c>
+      <c r="H6" s="37" t="n">
+        <v>168.75</v>
+      </c>
+      <c r="I6" s="37" t="n">
+        <v>210.9375</v>
+      </c>
+      <c r="J6" s="37" t="n">
+        <v>230.625</v>
+      </c>
+      <c r="K6" s="37" t="n">
+        <v>247.5</v>
+      </c>
+      <c r="L6" s="37" t="n">
+        <v>258.75</v>
+      </c>
+      <c r="M6" s="37" t="n">
+        <v>286.875</v>
+      </c>
+      <c r="N6" s="37" t="n">
+        <v>316.40625</v>
+      </c>
+      <c r="O6" s="37" t="n">
+        <v>337.5</v>
+      </c>
+      <c r="P6" s="37" t="n">
+        <v>358.59375</v>
+      </c>
+      <c r="Q6" s="37" t="n">
+        <v>371.25</v>
+      </c>
+      <c r="R6" s="37" t="n">
+        <v>379.6875</v>
+      </c>
+      <c r="S6" s="37" t="n">
+        <v>379.6875</v>
+      </c>
+      <c r="U6" s="38" t="n">
+        <v>379.6875</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="36" t="inlineStr">
+        <is>
+          <t>Ingresos (22,03 B2B / 22,22 B2C)</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>1340.28984375</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>1994.85</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>2431.2234375</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>2774.08828125</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>3740.34375</v>
+      </c>
+      <c r="I7" s="5" t="n">
+        <v>4675.4296875</v>
+      </c>
+      <c r="J7" s="5" t="n">
+        <v>5111.803124999999</v>
+      </c>
+      <c r="K7" s="5" t="n">
+        <v>5485.8375</v>
+      </c>
+      <c r="L7" s="5" t="n">
+        <v>5735.193749999999</v>
+      </c>
+      <c r="M7" s="5" t="n">
+        <v>6358.584374999999</v>
+      </c>
+      <c r="N7" s="5" t="n">
+        <v>7013.14453125</v>
+      </c>
+      <c r="O7" s="5" t="n">
+        <v>7480.6875</v>
+      </c>
+      <c r="P7" s="5" t="n">
+        <v>7948.23046875</v>
+      </c>
+      <c r="Q7" s="5" t="n">
+        <v>8228.75625</v>
+      </c>
+      <c r="R7" s="5" t="n">
+        <v>8415.7734375</v>
+      </c>
+      <c r="S7" s="5" t="n">
+        <v>8415.7734375</v>
+      </c>
+      <c r="U7" s="39" t="n">
+        <v>87150.00937499999</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="36" t="inlineStr">
+        <is>
+          <t>— Costes laborales empl.</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>-0</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>-0</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>-1753.345243393333</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>-1753.345243393333</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>-1753.345243393333</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>-1753.345243393333</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>-3506.690486786666</v>
+      </c>
+      <c r="I8" s="5" t="n">
+        <v>-3506.690486786666</v>
+      </c>
+      <c r="J8" s="5" t="n">
+        <v>-3506.690486786666</v>
+      </c>
+      <c r="K8" s="5" t="n">
+        <v>-3506.690486786666</v>
+      </c>
+      <c r="L8" s="5" t="n">
+        <v>-3506.690486786666</v>
+      </c>
+      <c r="M8" s="5" t="n">
+        <v>-5260.03573018</v>
+      </c>
+      <c r="N8" s="5" t="n">
+        <v>-5260.03573018</v>
+      </c>
+      <c r="O8" s="5" t="n">
+        <v>-5260.03573018</v>
+      </c>
+      <c r="P8" s="5" t="n">
+        <v>-5260.03573018</v>
+      </c>
+      <c r="Q8" s="5" t="n">
+        <v>-5260.03573018</v>
+      </c>
+      <c r="R8" s="5" t="n">
+        <v>-5260.03573018</v>
+      </c>
+      <c r="S8" s="5" t="n">
+        <v>-5260.03573018</v>
+      </c>
+      <c r="U8" s="39" t="n">
+        <v>-61367.08351876664</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="36" t="inlineStr">
+        <is>
+          <t>— Cuota autónomo titular</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>-80</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>-80</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>-80</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>-80</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>-80</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>-80</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>-160</v>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>-160</v>
+      </c>
+      <c r="J9" s="5" t="n">
+        <v>-160</v>
+      </c>
+      <c r="K9" s="5" t="n">
+        <v>-160</v>
+      </c>
+      <c r="L9" s="5" t="n">
+        <v>-160</v>
+      </c>
+      <c r="M9" s="5" t="n">
+        <v>-160</v>
+      </c>
+      <c r="N9" s="5" t="n">
+        <v>-320</v>
+      </c>
+      <c r="O9" s="5" t="n">
+        <v>-320</v>
+      </c>
+      <c r="P9" s="5" t="n">
+        <v>-320</v>
+      </c>
+      <c r="Q9" s="5" t="n">
+        <v>-320</v>
+      </c>
+      <c r="R9" s="5" t="n">
+        <v>-320</v>
+      </c>
+      <c r="S9" s="5" t="n">
+        <v>-320</v>
+      </c>
+      <c r="U9" s="39" t="n">
+        <v>-3360</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="36" t="inlineStr">
+        <is>
+          <t>— Materiales y transporte</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>-0</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>-0</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>-45.65390624999999</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>-67.94999999999999</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>-82.81406249999999</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>-94.49296874999999</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>-127.40625</v>
+      </c>
+      <c r="I10" s="5" t="n">
+        <v>-159.2578125</v>
+      </c>
+      <c r="J10" s="5" t="n">
+        <v>-174.121875</v>
+      </c>
+      <c r="K10" s="5" t="n">
+        <v>-186.8625</v>
+      </c>
+      <c r="L10" s="5" t="n">
+        <v>-195.35625</v>
+      </c>
+      <c r="M10" s="5" t="n">
+        <v>-216.590625</v>
+      </c>
+      <c r="N10" s="5" t="n">
+        <v>-238.88671875</v>
+      </c>
+      <c r="O10" s="5" t="n">
+        <v>-254.8125</v>
+      </c>
+      <c r="P10" s="5" t="n">
+        <v>-270.7382812499999</v>
+      </c>
+      <c r="Q10" s="5" t="n">
+        <v>-280.29375</v>
+      </c>
+      <c r="R10" s="5" t="n">
+        <v>-286.6640624999999</v>
+      </c>
+      <c r="S10" s="5" t="n">
+        <v>-286.6640624999999</v>
+      </c>
+      <c r="U10" s="39" t="n">
+        <v>-2968.565625</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="36" t="inlineStr">
+        <is>
+          <t>— Estructura (1430 €/mes)</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>-1430</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>-1430</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>-1430</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>-1430</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>-1430</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>-1430</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>-1430</v>
+      </c>
+      <c r="I11" s="5" t="n">
+        <v>-1430</v>
+      </c>
+      <c r="J11" s="5" t="n">
+        <v>-1430</v>
+      </c>
+      <c r="K11" s="5" t="n">
+        <v>-1430</v>
+      </c>
+      <c r="L11" s="5" t="n">
+        <v>-1430</v>
+      </c>
+      <c r="M11" s="5" t="n">
+        <v>-1430</v>
+      </c>
+      <c r="N11" s="5" t="n">
+        <v>-1430</v>
+      </c>
+      <c r="O11" s="5" t="n">
+        <v>-1430</v>
+      </c>
+      <c r="P11" s="5" t="n">
+        <v>-1430</v>
+      </c>
+      <c r="Q11" s="5" t="n">
+        <v>-1430</v>
+      </c>
+      <c r="R11" s="5" t="n">
+        <v>-1430</v>
+      </c>
+      <c r="S11" s="5" t="n">
+        <v>-1430</v>
+      </c>
+      <c r="U11" s="39" t="n">
+        <v>-25740</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="40" t="inlineStr">
+        <is>
+          <t>EBITDA MENSUAL</t>
+        </is>
+      </c>
+      <c r="B12" s="41" t="n">
+        <v>-1510</v>
+      </c>
+      <c r="C12" s="41" t="n">
+        <v>-1510</v>
+      </c>
+      <c r="D12" s="41" t="n">
+        <v>-1968.709305893333</v>
+      </c>
+      <c r="E12" s="41" t="n">
+        <v>-1336.445243393333</v>
+      </c>
+      <c r="F12" s="41" t="n">
+        <v>-914.9358683933334</v>
+      </c>
+      <c r="G12" s="41" t="n">
+        <v>-583.7499308933334</v>
+      </c>
+      <c r="H12" s="41" t="n">
+        <v>-1483.752986786666</v>
+      </c>
+      <c r="I12" s="41" t="n">
+        <v>-580.5186117866665</v>
+      </c>
+      <c r="J12" s="41" t="n">
+        <v>-159.0092367866671</v>
+      </c>
+      <c r="K12" s="42" t="n">
+        <v>202.2845132133332</v>
+      </c>
+      <c r="L12" s="42" t="n">
+        <v>443.1470132133329</v>
+      </c>
+      <c r="M12" s="41" t="n">
+        <v>-708.04198018</v>
+      </c>
+      <c r="N12" s="41" t="n">
+        <v>-235.7779176799995</v>
+      </c>
+      <c r="O12" s="42" t="n">
+        <v>215.8392698200005</v>
+      </c>
+      <c r="P12" s="42" t="n">
+        <v>667.4564573200005</v>
+      </c>
+      <c r="Q12" s="42" t="n">
+        <v>938.426769820001</v>
+      </c>
+      <c r="R12" s="42" t="n">
+        <v>1119.07364482</v>
+      </c>
+      <c r="S12" s="42" t="n">
+        <v>1119.07364482</v>
+      </c>
+      <c r="U12" s="39" t="n">
+        <v>-6285.639768766665</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="40" t="inlineStr">
+        <is>
+          <t>FLUJO ACUMULADO</t>
+        </is>
+      </c>
+      <c r="B13" s="50" t="n">
+        <v>-4310</v>
+      </c>
+      <c r="C13" s="50" t="n">
+        <v>-5820</v>
+      </c>
+      <c r="D13" s="50" t="n">
+        <v>-7788.709305893333</v>
+      </c>
+      <c r="E13" s="50" t="n">
+        <v>-9125.154549286666</v>
+      </c>
+      <c r="F13" s="50" t="n">
+        <v>-10040.09041768</v>
+      </c>
+      <c r="G13" s="50" t="n">
+        <v>-10623.84034857333</v>
+      </c>
+      <c r="H13" s="50" t="n">
+        <v>-12107.59333536</v>
+      </c>
+      <c r="I13" s="50" t="n">
+        <v>-12688.11194714667</v>
+      </c>
+      <c r="J13" s="50" t="n">
+        <v>-12847.12118393333</v>
+      </c>
+      <c r="K13" s="50" t="n">
+        <v>-12644.83667072</v>
+      </c>
+      <c r="L13" s="50" t="n">
+        <v>-12201.68965750667</v>
+      </c>
+      <c r="M13" s="50" t="n">
+        <v>-12909.73163768667</v>
+      </c>
+      <c r="N13" s="50" t="n">
+        <v>-13145.50955536667</v>
+      </c>
+      <c r="O13" s="50" t="n">
+        <v>-12929.67028554667</v>
+      </c>
+      <c r="P13" s="50" t="n">
+        <v>-12262.21382822667</v>
+      </c>
+      <c r="Q13" s="50" t="n">
+        <v>-11323.78705840667</v>
+      </c>
+      <c r="R13" s="50" t="n">
+        <v>-10204.71341358667</v>
+      </c>
+      <c r="S13" s="50" t="n">
+        <v>-9085.639768766665</v>
+      </c>
+      <c r="U13" s="39" t="n">
+        <v>-9085.639768766665</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ✅ Capital necesario: 13146 € mín. | Rec. con +25%: 16432 €  | 1er mes positivo: M10  | BEP acumulado: &gt;M18</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="31" t="inlineStr">
+        <is>
+          <t>ESCENARIO B – LEAN: home office + coche propio  ★ RECOMENDADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>INVERSIÓN INICIAL (setup)</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="n">
+        <v>-800</v>
+      </c>
+      <c r="C25" s="45" t="inlineStr"/>
+      <c r="D25" s="45" t="inlineStr"/>
+      <c r="E25" s="45" t="inlineStr"/>
+      <c r="F25" s="45" t="inlineStr"/>
+      <c r="G25" s="45" t="inlineStr"/>
+      <c r="H25" s="45" t="inlineStr"/>
+      <c r="I25" s="45" t="inlineStr"/>
+      <c r="J25" s="45" t="inlineStr"/>
+      <c r="K25" s="45" t="inlineStr"/>
+      <c r="L25" s="45" t="inlineStr"/>
+      <c r="M25" s="45" t="inlineStr"/>
+      <c r="N25" s="45" t="inlineStr"/>
+      <c r="O25" s="45" t="inlineStr"/>
+      <c r="P25" s="45" t="inlineStr"/>
+      <c r="Q25" s="45" t="inlineStr"/>
+      <c r="R25" s="45" t="inlineStr"/>
+      <c r="S25" s="45" t="inlineStr"/>
+      <c r="T25" s="45" t="inlineStr"/>
+      <c r="U25" s="45" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="51" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="B26" s="33" t="inlineStr">
+        <is>
+          <t>Jul'26</t>
+        </is>
+      </c>
+      <c r="C26" s="33" t="inlineStr">
+        <is>
+          <t>Ago'26</t>
+        </is>
+      </c>
+      <c r="D26" s="33" t="inlineStr">
+        <is>
+          <t>Sep'26</t>
+        </is>
+      </c>
+      <c r="E26" s="33" t="inlineStr">
+        <is>
+          <t>Oct'26</t>
+        </is>
+      </c>
+      <c r="F26" s="33" t="inlineStr">
+        <is>
+          <t>Nov'26</t>
+        </is>
+      </c>
+      <c r="G26" s="33" t="inlineStr">
+        <is>
+          <t>Dic'26</t>
+        </is>
+      </c>
+      <c r="H26" s="33" t="inlineStr">
+        <is>
+          <t>Ene'27</t>
+        </is>
+      </c>
+      <c r="I26" s="33" t="inlineStr">
+        <is>
+          <t>Feb'27</t>
+        </is>
+      </c>
+      <c r="J26" s="33" t="inlineStr">
+        <is>
+          <t>Mar'27</t>
+        </is>
+      </c>
+      <c r="K26" s="33" t="inlineStr">
+        <is>
+          <t>Abr'27</t>
+        </is>
+      </c>
+      <c r="L26" s="33" t="inlineStr">
+        <is>
+          <t>May'27</t>
+        </is>
+      </c>
+      <c r="M26" s="33" t="inlineStr">
+        <is>
+          <t>Jun'27</t>
+        </is>
+      </c>
+      <c r="N26" s="33" t="inlineStr">
+        <is>
+          <t>Jul'27</t>
+        </is>
+      </c>
+      <c r="O26" s="33" t="inlineStr">
+        <is>
+          <t>Ago'27</t>
+        </is>
+      </c>
+      <c r="P26" s="33" t="inlineStr">
+        <is>
+          <t>Sep'27</t>
+        </is>
+      </c>
+      <c r="Q26" s="33" t="inlineStr">
+        <is>
+          <t>Oct'27</t>
+        </is>
+      </c>
+      <c r="R26" s="33" t="inlineStr">
+        <is>
+          <t>Nov'27</t>
+        </is>
+      </c>
+      <c r="S26" s="33" t="inlineStr">
+        <is>
+          <t>Dic'27</t>
+        </is>
+      </c>
+      <c r="U26" s="47" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="36" t="inlineStr">
+        <is>
+          <t>Nº empleados activos</t>
+        </is>
+      </c>
+      <c r="B27" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="H27" s="48" t="n">
+        <v>2</v>
+      </c>
+      <c r="I27" s="48" t="n">
+        <v>2</v>
+      </c>
+      <c r="J27" s="48" t="n">
+        <v>2</v>
+      </c>
+      <c r="K27" s="48" t="n">
+        <v>2</v>
+      </c>
+      <c r="L27" s="48" t="n">
+        <v>2</v>
+      </c>
+      <c r="M27" s="48" t="n">
+        <v>3</v>
+      </c>
+      <c r="N27" s="48" t="n">
+        <v>3</v>
+      </c>
+      <c r="O27" s="48" t="n">
+        <v>3</v>
+      </c>
+      <c r="P27" s="48" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q27" s="48" t="n">
+        <v>3</v>
+      </c>
+      <c r="R27" s="48" t="n">
+        <v>3</v>
+      </c>
+      <c r="S27" s="48" t="n">
+        <v>3</v>
+      </c>
+      <c r="U27" s="49" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="36" t="inlineStr">
+        <is>
+          <t>Horas facturadas/mes</t>
+        </is>
+      </c>
+      <c r="B28" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="37" t="n">
+        <v>60.46875</v>
+      </c>
+      <c r="E28" s="37" t="n">
+        <v>90</v>
+      </c>
+      <c r="F28" s="37" t="n">
+        <v>109.6875</v>
+      </c>
+      <c r="G28" s="37" t="n">
+        <v>125.15625</v>
+      </c>
+      <c r="H28" s="37" t="n">
+        <v>168.75</v>
+      </c>
+      <c r="I28" s="37" t="n">
+        <v>210.9375</v>
+      </c>
+      <c r="J28" s="37" t="n">
+        <v>230.625</v>
+      </c>
+      <c r="K28" s="37" t="n">
+        <v>247.5</v>
+      </c>
+      <c r="L28" s="37" t="n">
+        <v>258.75</v>
+      </c>
+      <c r="M28" s="37" t="n">
+        <v>286.875</v>
+      </c>
+      <c r="N28" s="37" t="n">
+        <v>316.40625</v>
+      </c>
+      <c r="O28" s="37" t="n">
+        <v>337.5</v>
+      </c>
+      <c r="P28" s="37" t="n">
+        <v>358.59375</v>
+      </c>
+      <c r="Q28" s="37" t="n">
+        <v>371.25</v>
+      </c>
+      <c r="R28" s="37" t="n">
+        <v>379.6875</v>
+      </c>
+      <c r="S28" s="37" t="n">
+        <v>379.6875</v>
+      </c>
+      <c r="U28" s="38" t="n">
+        <v>379.6875</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="36" t="inlineStr">
+        <is>
+          <t>Ingresos (22,03 B2B / 22,22 B2C)</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="5" t="n">
+        <v>1340.28984375</v>
+      </c>
+      <c r="E29" s="5" t="n">
+        <v>1994.85</v>
+      </c>
+      <c r="F29" s="5" t="n">
+        <v>2431.2234375</v>
+      </c>
+      <c r="G29" s="5" t="n">
+        <v>2774.08828125</v>
+      </c>
+      <c r="H29" s="5" t="n">
+        <v>3740.34375</v>
+      </c>
+      <c r="I29" s="5" t="n">
+        <v>4675.4296875</v>
+      </c>
+      <c r="J29" s="5" t="n">
+        <v>5111.803124999999</v>
+      </c>
+      <c r="K29" s="5" t="n">
+        <v>5485.8375</v>
+      </c>
+      <c r="L29" s="5" t="n">
+        <v>5735.193749999999</v>
+      </c>
+      <c r="M29" s="5" t="n">
+        <v>6358.584374999999</v>
+      </c>
+      <c r="N29" s="5" t="n">
+        <v>7013.14453125</v>
+      </c>
+      <c r="O29" s="5" t="n">
+        <v>7480.6875</v>
+      </c>
+      <c r="P29" s="5" t="n">
+        <v>7948.23046875</v>
+      </c>
+      <c r="Q29" s="5" t="n">
+        <v>8228.75625</v>
+      </c>
+      <c r="R29" s="5" t="n">
+        <v>8415.7734375</v>
+      </c>
+      <c r="S29" s="5" t="n">
+        <v>8415.7734375</v>
+      </c>
+      <c r="U29" s="39" t="n">
+        <v>87150.00937499999</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="36" t="inlineStr">
+        <is>
+          <t>— Costes laborales empl.</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>-0</v>
+      </c>
+      <c r="C30" s="5" t="n">
+        <v>-0</v>
+      </c>
+      <c r="D30" s="5" t="n">
+        <v>-1753.345243393333</v>
+      </c>
+      <c r="E30" s="5" t="n">
+        <v>-1753.345243393333</v>
+      </c>
+      <c r="F30" s="5" t="n">
+        <v>-1753.345243393333</v>
+      </c>
+      <c r="G30" s="5" t="n">
+        <v>-1753.345243393333</v>
+      </c>
+      <c r="H30" s="5" t="n">
+        <v>-3506.690486786666</v>
+      </c>
+      <c r="I30" s="5" t="n">
+        <v>-3506.690486786666</v>
+      </c>
+      <c r="J30" s="5" t="n">
+        <v>-3506.690486786666</v>
+      </c>
+      <c r="K30" s="5" t="n">
+        <v>-3506.690486786666</v>
+      </c>
+      <c r="L30" s="5" t="n">
+        <v>-3506.690486786666</v>
+      </c>
+      <c r="M30" s="5" t="n">
+        <v>-5260.03573018</v>
+      </c>
+      <c r="N30" s="5" t="n">
+        <v>-5260.03573018</v>
+      </c>
+      <c r="O30" s="5" t="n">
+        <v>-5260.03573018</v>
+      </c>
+      <c r="P30" s="5" t="n">
+        <v>-5260.03573018</v>
+      </c>
+      <c r="Q30" s="5" t="n">
+        <v>-5260.03573018</v>
+      </c>
+      <c r="R30" s="5" t="n">
+        <v>-5260.03573018</v>
+      </c>
+      <c r="S30" s="5" t="n">
+        <v>-5260.03573018</v>
+      </c>
+      <c r="U30" s="39" t="n">
+        <v>-61367.08351876664</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="36" t="inlineStr">
+        <is>
+          <t>— Cuota autónomo titular</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>-80</v>
+      </c>
+      <c r="C31" s="5" t="n">
+        <v>-80</v>
+      </c>
+      <c r="D31" s="5" t="n">
+        <v>-80</v>
+      </c>
+      <c r="E31" s="5" t="n">
+        <v>-80</v>
+      </c>
+      <c r="F31" s="5" t="n">
+        <v>-80</v>
+      </c>
+      <c r="G31" s="5" t="n">
+        <v>-80</v>
+      </c>
+      <c r="H31" s="5" t="n">
+        <v>-160</v>
+      </c>
+      <c r="I31" s="5" t="n">
+        <v>-160</v>
+      </c>
+      <c r="J31" s="5" t="n">
+        <v>-160</v>
+      </c>
+      <c r="K31" s="5" t="n">
+        <v>-160</v>
+      </c>
+      <c r="L31" s="5" t="n">
+        <v>-160</v>
+      </c>
+      <c r="M31" s="5" t="n">
+        <v>-160</v>
+      </c>
+      <c r="N31" s="5" t="n">
+        <v>-320</v>
+      </c>
+      <c r="O31" s="5" t="n">
+        <v>-320</v>
+      </c>
+      <c r="P31" s="5" t="n">
+        <v>-320</v>
+      </c>
+      <c r="Q31" s="5" t="n">
+        <v>-320</v>
+      </c>
+      <c r="R31" s="5" t="n">
+        <v>-320</v>
+      </c>
+      <c r="S31" s="5" t="n">
+        <v>-320</v>
+      </c>
+      <c r="U31" s="39" t="n">
+        <v>-3360</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="36" t="inlineStr">
+        <is>
+          <t>— Materiales y transporte</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>-0</v>
+      </c>
+      <c r="C32" s="5" t="n">
+        <v>-0</v>
+      </c>
+      <c r="D32" s="5" t="n">
+        <v>-45.65390624999999</v>
+      </c>
+      <c r="E32" s="5" t="n">
+        <v>-67.94999999999999</v>
+      </c>
+      <c r="F32" s="5" t="n">
+        <v>-82.81406249999999</v>
+      </c>
+      <c r="G32" s="5" t="n">
+        <v>-94.49296874999999</v>
+      </c>
+      <c r="H32" s="5" t="n">
+        <v>-127.40625</v>
+      </c>
+      <c r="I32" s="5" t="n">
+        <v>-159.2578125</v>
+      </c>
+      <c r="J32" s="5" t="n">
+        <v>-174.121875</v>
+      </c>
+      <c r="K32" s="5" t="n">
+        <v>-186.8625</v>
+      </c>
+      <c r="L32" s="5" t="n">
+        <v>-195.35625</v>
+      </c>
+      <c r="M32" s="5" t="n">
+        <v>-216.590625</v>
+      </c>
+      <c r="N32" s="5" t="n">
+        <v>-238.88671875</v>
+      </c>
+      <c r="O32" s="5" t="n">
+        <v>-254.8125</v>
+      </c>
+      <c r="P32" s="5" t="n">
+        <v>-270.7382812499999</v>
+      </c>
+      <c r="Q32" s="5" t="n">
+        <v>-280.29375</v>
+      </c>
+      <c r="R32" s="5" t="n">
+        <v>-286.6640624999999</v>
+      </c>
+      <c r="S32" s="5" t="n">
+        <v>-286.6640624999999</v>
+      </c>
+      <c r="U32" s="39" t="n">
+        <v>-2968.565625</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="36" t="inlineStr">
+        <is>
+          <t>— Estructura (780 €/mes)</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>-780</v>
+      </c>
+      <c r="C33" s="5" t="n">
+        <v>-780</v>
+      </c>
+      <c r="D33" s="5" t="n">
+        <v>-780</v>
+      </c>
+      <c r="E33" s="5" t="n">
+        <v>-780</v>
+      </c>
+      <c r="F33" s="5" t="n">
+        <v>-780</v>
+      </c>
+      <c r="G33" s="5" t="n">
+        <v>-780</v>
+      </c>
+      <c r="H33" s="5" t="n">
+        <v>-780</v>
+      </c>
+      <c r="I33" s="5" t="n">
+        <v>-780</v>
+      </c>
+      <c r="J33" s="5" t="n">
+        <v>-780</v>
+      </c>
+      <c r="K33" s="5" t="n">
+        <v>-780</v>
+      </c>
+      <c r="L33" s="5" t="n">
+        <v>-780</v>
+      </c>
+      <c r="M33" s="5" t="n">
+        <v>-780</v>
+      </c>
+      <c r="N33" s="5" t="n">
+        <v>-780</v>
+      </c>
+      <c r="O33" s="5" t="n">
+        <v>-780</v>
+      </c>
+      <c r="P33" s="5" t="n">
+        <v>-780</v>
+      </c>
+      <c r="Q33" s="5" t="n">
+        <v>-780</v>
+      </c>
+      <c r="R33" s="5" t="n">
+        <v>-780</v>
+      </c>
+      <c r="S33" s="5" t="n">
+        <v>-780</v>
+      </c>
+      <c r="U33" s="39" t="n">
+        <v>-14040</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="40" t="inlineStr">
+        <is>
+          <t>EBITDA MENSUAL</t>
+        </is>
+      </c>
+      <c r="B34" s="41" t="n">
+        <v>-860</v>
+      </c>
+      <c r="C34" s="41" t="n">
+        <v>-860</v>
+      </c>
+      <c r="D34" s="41" t="n">
+        <v>-1318.709305893333</v>
+      </c>
+      <c r="E34" s="41" t="n">
+        <v>-686.4452433933334</v>
+      </c>
+      <c r="F34" s="41" t="n">
+        <v>-264.9358683933334</v>
+      </c>
+      <c r="G34" s="42" t="n">
+        <v>66.25006910666661</v>
+      </c>
+      <c r="H34" s="41" t="n">
+        <v>-833.7529867866665</v>
+      </c>
+      <c r="I34" s="42" t="n">
+        <v>69.4813882133335</v>
+      </c>
+      <c r="J34" s="42" t="n">
+        <v>490.9907632133329</v>
+      </c>
+      <c r="K34" s="42" t="n">
+        <v>852.2845132133332</v>
+      </c>
+      <c r="L34" s="42" t="n">
+        <v>1093.147013213333</v>
+      </c>
+      <c r="M34" s="41" t="n">
+        <v>-58.04198018</v>
+      </c>
+      <c r="N34" s="42" t="n">
+        <v>414.2220823200005</v>
+      </c>
+      <c r="O34" s="42" t="n">
+        <v>865.8392698200005</v>
+      </c>
+      <c r="P34" s="42" t="n">
+        <v>1317.45645732</v>
+      </c>
+      <c r="Q34" s="42" t="n">
+        <v>1588.426769820001</v>
+      </c>
+      <c r="R34" s="42" t="n">
+        <v>1769.07364482</v>
+      </c>
+      <c r="S34" s="42" t="n">
+        <v>1769.07364482</v>
+      </c>
+      <c r="U34" s="39" t="n">
+        <v>5414.360231233336</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="40" t="inlineStr">
+        <is>
+          <t>FLUJO ACUMULADO</t>
+        </is>
+      </c>
+      <c r="B35" s="50" t="n">
+        <v>-1660</v>
+      </c>
+      <c r="C35" s="50" t="n">
+        <v>-2520</v>
+      </c>
+      <c r="D35" s="50" t="n">
+        <v>-3838.709305893333</v>
+      </c>
+      <c r="E35" s="50" t="n">
+        <v>-4525.154549286666</v>
+      </c>
+      <c r="F35" s="50" t="n">
+        <v>-4790.09041768</v>
+      </c>
+      <c r="G35" s="50" t="n">
+        <v>-4723.840348573332</v>
+      </c>
+      <c r="H35" s="50" t="n">
+        <v>-5557.593335359999</v>
+      </c>
+      <c r="I35" s="50" t="n">
+        <v>-5488.111947146666</v>
+      </c>
+      <c r="J35" s="50" t="n">
+        <v>-4997.121183933334</v>
+      </c>
+      <c r="K35" s="50" t="n">
+        <v>-4144.83667072</v>
+      </c>
+      <c r="L35" s="50" t="n">
+        <v>-3051.689657506668</v>
+      </c>
+      <c r="M35" s="50" t="n">
+        <v>-3109.731637686667</v>
+      </c>
+      <c r="N35" s="50" t="n">
+        <v>-2695.509555366667</v>
+      </c>
+      <c r="O35" s="50" t="n">
+        <v>-1829.670285546666</v>
+      </c>
+      <c r="P35" s="50" t="n">
+        <v>-512.213828226666</v>
+      </c>
+      <c r="Q35" s="52" t="n">
+        <v>1076.212941593335</v>
+      </c>
+      <c r="R35" s="52" t="n">
+        <v>2845.286586413335</v>
+      </c>
+      <c r="S35" s="52" t="n">
+        <v>4614.360231233336</v>
+      </c>
+      <c r="U35" s="39" t="n">
+        <v>4614.360231233336</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ✅ Capital necesario: 5558 € mín. | Rec. con +25%: 6947 €  | 1er mes positivo: M6  | BEP acumulado: M16</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A24:U24"/>
+    <mergeCell ref="A36:U36"/>
+    <mergeCell ref="A14:U14"/>
+    <mergeCell ref="A2:U2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>